<commit_message>
add bulk density data
</commit_message>
<xml_diff>
--- a/data/Field_soil_moisture.xlsx
+++ b/data/Field_soil_moisture.xlsx
@@ -1,21 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10621"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10628"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/andiemartinez/Desktop/Metagenomic_Project/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9B556EB-8104-8040-8C88-0A5571C91739}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D6564A4-EF1A-5542-946D-A0B3DACD2D3C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1160" yWindow="500" windowWidth="27240" windowHeight="15280" activeTab="2" xr2:uid="{FE8B7330-86A3-ED4C-8E2C-DB45F152A5F6}"/>
+    <workbookView xWindow="1560" yWindow="500" windowWidth="27240" windowHeight="15280" activeTab="3" xr2:uid="{FE8B7330-86A3-ED4C-8E2C-DB45F152A5F6}"/>
   </bookViews>
   <sheets>
     <sheet name="T1_sieved" sheetId="1" r:id="rId1"/>
     <sheet name="T2_sieved" sheetId="2" r:id="rId2"/>
     <sheet name="T2_unsieved" sheetId="3" r:id="rId3"/>
+    <sheet name="bulk_density" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -88,7 +89,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="422" uniqueCount="171">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="415" uniqueCount="176">
   <si>
     <t>sample</t>
   </si>
@@ -601,6 +602,21 @@
   </si>
   <si>
     <t>IV</t>
+  </si>
+  <si>
+    <t>10 cores</t>
+  </si>
+  <si>
+    <t>notes</t>
+  </si>
+  <si>
+    <t>tray(g)</t>
+  </si>
+  <si>
+    <t>tray+moist_soil(g)</t>
+  </si>
+  <si>
+    <t>moist_soil(g)</t>
   </si>
 </sst>
 </file>
@@ -7038,7 +7054,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{681446B1-FAED-1D4A-8EC9-22E0992AE038}">
-  <dimension ref="A1:K73"/>
+  <dimension ref="A1:K61"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="5" width="13.5" customWidth="1"/>
@@ -7119,8 +7135,20 @@
       <c r="G2" s="1">
         <v>27.07</v>
       </c>
+      <c r="H2">
+        <f>G2-F2</f>
+        <v>24.61</v>
+      </c>
       <c r="I2" s="1">
         <v>22.96</v>
+      </c>
+      <c r="J2">
+        <f>I2-F2</f>
+        <v>20.5</v>
+      </c>
+      <c r="K2">
+        <f>J2/H2*100</f>
+        <v>83.299471759447385</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.2">
@@ -7160,8 +7188,20 @@
       <c r="G3" s="1">
         <v>25.01</v>
       </c>
+      <c r="H3">
+        <f t="shared" ref="H3:H54" si="0">G3-F3</f>
+        <v>22.42</v>
+      </c>
       <c r="I3" s="1">
         <v>21.2</v>
+      </c>
+      <c r="J3">
+        <f t="shared" ref="J3:J54" si="1">I3-F3</f>
+        <v>18.61</v>
+      </c>
+      <c r="K3">
+        <f t="shared" ref="K3:K54" si="2">J3/H3*100</f>
+        <v>83.006244424620874</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.2">
@@ -7201,8 +7241,20 @@
       <c r="G4" s="1">
         <v>27.13</v>
       </c>
+      <c r="H4">
+        <f t="shared" si="0"/>
+        <v>24.45</v>
+      </c>
       <c r="I4" s="1">
         <v>21.81</v>
+      </c>
+      <c r="J4">
+        <f t="shared" si="1"/>
+        <v>19.13</v>
+      </c>
+      <c r="K4">
+        <f t="shared" si="2"/>
+        <v>78.241308793456028</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.2">
@@ -7242,13 +7294,25 @@
       <c r="G5" s="1">
         <v>25.77</v>
       </c>
+      <c r="H5">
+        <f t="shared" si="0"/>
+        <v>23.07</v>
+      </c>
       <c r="I5" s="1">
         <v>21.35</v>
       </c>
+      <c r="J5">
+        <f t="shared" si="1"/>
+        <v>18.650000000000002</v>
+      </c>
+      <c r="K5">
+        <f t="shared" si="2"/>
+        <v>80.840918942349376</v>
+      </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="C6" t="str" cm="1">
         <f t="array" ref="C6">_xlfn.IFS(
@@ -7275,12 +7339,33 @@
 ISNUMBER(SEARCH("RCL*",A6)),"RCL",
 ISNUMBER(SEARCH("SWW*",A6)),"SWW",
 ISNUMBER(SEARCH("MNHV*",A6)),"MNHV")</f>
-        <v>C1</v>
+        <v>MNHV</v>
+      </c>
+      <c r="F6" s="1">
+        <v>2.46</v>
+      </c>
+      <c r="G6" s="1">
+        <v>28.37</v>
+      </c>
+      <c r="H6">
+        <f t="shared" si="0"/>
+        <v>25.91</v>
+      </c>
+      <c r="I6" s="1">
+        <v>23.6</v>
+      </c>
+      <c r="J6">
+        <f t="shared" si="1"/>
+        <v>21.14</v>
+      </c>
+      <c r="K6">
+        <f t="shared" si="2"/>
+        <v>81.590119644924741</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="C7" t="str" cm="1">
         <f t="array" ref="C7">_xlfn.IFS(
@@ -7307,12 +7392,33 @@
 ISNUMBER(SEARCH("RCL*",A7)),"RCL",
 ISNUMBER(SEARCH("SWW*",A7)),"SWW",
 ISNUMBER(SEARCH("MNHV*",A7)),"MNHV")</f>
-        <v>C1</v>
+        <v>MNHV</v>
+      </c>
+      <c r="F7" s="1">
+        <v>2.63</v>
+      </c>
+      <c r="G7" s="1">
+        <v>25.92</v>
+      </c>
+      <c r="H7">
+        <f t="shared" si="0"/>
+        <v>23.290000000000003</v>
+      </c>
+      <c r="I7" s="1">
+        <v>21.93</v>
+      </c>
+      <c r="J7">
+        <f t="shared" si="1"/>
+        <v>19.3</v>
+      </c>
+      <c r="K7">
+        <f t="shared" si="2"/>
+        <v>82.868183769858305</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="C8" t="str" cm="1">
         <f t="array" ref="C8">_xlfn.IFS(
@@ -7339,12 +7445,33 @@
 ISNUMBER(SEARCH("RCL*",A8)),"RCL",
 ISNUMBER(SEARCH("SWW*",A8)),"SWW",
 ISNUMBER(SEARCH("MNHV*",A8)),"MNHV")</f>
-        <v>C2</v>
+        <v>ORG</v>
+      </c>
+      <c r="F8" s="1">
+        <v>2.64</v>
+      </c>
+      <c r="G8" s="1">
+        <v>26.06</v>
+      </c>
+      <c r="H8">
+        <f t="shared" si="0"/>
+        <v>23.419999999999998</v>
+      </c>
+      <c r="I8" s="1">
+        <v>22.12</v>
+      </c>
+      <c r="J8">
+        <f t="shared" si="1"/>
+        <v>19.48</v>
+      </c>
+      <c r="K8">
+        <f t="shared" si="2"/>
+        <v>83.176771989752353</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="C9" t="str" cm="1">
         <f t="array" ref="C9">_xlfn.IFS(
@@ -7371,12 +7498,33 @@
 ISNUMBER(SEARCH("RCL*",A9)),"RCL",
 ISNUMBER(SEARCH("SWW*",A9)),"SWW",
 ISNUMBER(SEARCH("MNHV*",A9)),"MNHV")</f>
-        <v>C2</v>
+        <v>ORG</v>
+      </c>
+      <c r="F9" s="1">
+        <v>2.62</v>
+      </c>
+      <c r="G9" s="1">
+        <v>25.22</v>
+      </c>
+      <c r="H9">
+        <f t="shared" si="0"/>
+        <v>22.599999999999998</v>
+      </c>
+      <c r="I9" s="1">
+        <v>21.58</v>
+      </c>
+      <c r="J9">
+        <f t="shared" si="1"/>
+        <v>18.959999999999997</v>
+      </c>
+      <c r="K9">
+        <f t="shared" si="2"/>
+        <v>83.893805309734503</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="C10" t="str" cm="1">
         <f t="array" ref="C10">_xlfn.IFS(
@@ -7403,21 +7551,33 @@
 ISNUMBER(SEARCH("RCL*",A10)),"RCL",
 ISNUMBER(SEARCH("SWW*",A10)),"SWW",
 ISNUMBER(SEARCH("MNHV*",A10)),"MNHV")</f>
-        <v>MNHV</v>
+        <v>PRY</v>
       </c>
       <c r="F10" s="1">
-        <v>2.46</v>
+        <v>2.61</v>
       </c>
       <c r="G10" s="1">
-        <v>28.37</v>
+        <v>26.46</v>
+      </c>
+      <c r="H10">
+        <f t="shared" si="0"/>
+        <v>23.85</v>
       </c>
       <c r="I10" s="1">
-        <v>23.6</v>
+        <v>22.16</v>
+      </c>
+      <c r="J10">
+        <f t="shared" si="1"/>
+        <v>19.55</v>
+      </c>
+      <c r="K10">
+        <f t="shared" si="2"/>
+        <v>81.970649895178198</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="C11" t="str" cm="1">
         <f t="array" ref="C11">_xlfn.IFS(
@@ -7444,21 +7604,33 @@
 ISNUMBER(SEARCH("RCL*",A11)),"RCL",
 ISNUMBER(SEARCH("SWW*",A11)),"SWW",
 ISNUMBER(SEARCH("MNHV*",A11)),"MNHV")</f>
-        <v>MNHV</v>
+        <v>PRY</v>
       </c>
       <c r="F11" s="1">
-        <v>2.63</v>
+        <v>2.72</v>
       </c>
       <c r="G11" s="1">
-        <v>25.92</v>
+        <v>25.85</v>
+      </c>
+      <c r="H11">
+        <f t="shared" si="0"/>
+        <v>23.130000000000003</v>
       </c>
       <c r="I11" s="1">
-        <v>21.93</v>
+        <v>21.72</v>
+      </c>
+      <c r="J11">
+        <f t="shared" si="1"/>
+        <v>19</v>
+      </c>
+      <c r="K11">
+        <f t="shared" si="2"/>
+        <v>82.144401210549063</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="C12" t="str" cm="1">
         <f t="array" ref="C12">_xlfn.IFS(
@@ -7485,21 +7657,33 @@
 ISNUMBER(SEARCH("RCL*",A12)),"RCL",
 ISNUMBER(SEARCH("SWW*",A12)),"SWW",
 ISNUMBER(SEARCH("MNHV*",A12)),"MNHV")</f>
-        <v>ORG</v>
+        <v>RCL</v>
       </c>
       <c r="F12" s="1">
-        <v>2.64</v>
+        <v>2.77</v>
       </c>
       <c r="G12" s="1">
-        <v>26.06</v>
+        <v>29.39</v>
+      </c>
+      <c r="H12">
+        <f t="shared" si="0"/>
+        <v>26.62</v>
       </c>
       <c r="I12" s="1">
-        <v>22.12</v>
+        <v>24.01</v>
+      </c>
+      <c r="J12">
+        <f t="shared" si="1"/>
+        <v>21.240000000000002</v>
+      </c>
+      <c r="K12">
+        <f t="shared" si="2"/>
+        <v>79.789631855747572</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="C13" t="str" cm="1">
         <f t="array" ref="C13">_xlfn.IFS(
@@ -7526,21 +7710,33 @@
 ISNUMBER(SEARCH("RCL*",A13)),"RCL",
 ISNUMBER(SEARCH("SWW*",A13)),"SWW",
 ISNUMBER(SEARCH("MNHV*",A13)),"MNHV")</f>
-        <v>ORG</v>
+        <v>RCL</v>
       </c>
       <c r="F13" s="1">
-        <v>2.62</v>
+        <v>2.76</v>
       </c>
       <c r="G13" s="1">
-        <v>25.22</v>
+        <v>29.05</v>
+      </c>
+      <c r="H13">
+        <f t="shared" si="0"/>
+        <v>26.29</v>
       </c>
       <c r="I13" s="1">
-        <v>21.58</v>
+        <v>23.65</v>
+      </c>
+      <c r="J13">
+        <f t="shared" si="1"/>
+        <v>20.89</v>
+      </c>
+      <c r="K13">
+        <f t="shared" si="2"/>
+        <v>79.4598706732598</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="C14" t="str" cm="1">
         <f t="array" ref="C14">_xlfn.IFS(
@@ -7567,21 +7763,33 @@
 ISNUMBER(SEARCH("RCL*",A14)),"RCL",
 ISNUMBER(SEARCH("SWW*",A14)),"SWW",
 ISNUMBER(SEARCH("MNHV*",A14)),"MNHV")</f>
-        <v>PRY</v>
+        <v>SWW</v>
       </c>
       <c r="F14" s="1">
-        <v>2.61</v>
+        <v>2.7</v>
       </c>
       <c r="G14" s="1">
-        <v>26.46</v>
+        <v>25.75</v>
+      </c>
+      <c r="H14">
+        <f t="shared" si="0"/>
+        <v>23.05</v>
       </c>
       <c r="I14" s="1">
-        <v>22.16</v>
+        <v>21.23</v>
+      </c>
+      <c r="J14">
+        <f t="shared" si="1"/>
+        <v>18.53</v>
+      </c>
+      <c r="K14">
+        <f t="shared" si="2"/>
+        <v>80.39045553145337</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="C15" t="str" cm="1">
         <f t="array" ref="C15">_xlfn.IFS(
@@ -7608,21 +7816,33 @@
 ISNUMBER(SEARCH("RCL*",A15)),"RCL",
 ISNUMBER(SEARCH("SWW*",A15)),"SWW",
 ISNUMBER(SEARCH("MNHV*",A15)),"MNHV")</f>
-        <v>PRY</v>
+        <v>SWW</v>
       </c>
       <c r="F15" s="1">
-        <v>2.72</v>
+        <v>2.69</v>
       </c>
       <c r="G15" s="1">
-        <v>25.85</v>
+        <v>26.58</v>
+      </c>
+      <c r="H15">
+        <f t="shared" si="0"/>
+        <v>23.889999999999997</v>
       </c>
       <c r="I15" s="1">
-        <v>21.72</v>
+        <v>21.44</v>
+      </c>
+      <c r="J15">
+        <f t="shared" si="1"/>
+        <v>18.75</v>
+      </c>
+      <c r="K15">
+        <f t="shared" si="2"/>
+        <v>78.484721640853934</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="C16" t="str" cm="1">
         <f t="array" ref="C16">_xlfn.IFS(
@@ -7630,7 +7850,7 @@
 ISNUMBER(SEARCH("III*",A16)),"III",
 ISNUMBER(SEARCH("II*",A16)),"II",
 ISNUMBER(SEARCH("I*",A16)),"I")</f>
-        <v>III</v>
+        <v>I</v>
       </c>
       <c r="D16" cm="1">
         <f t="array" ref="D16">_xlfn.IFS(
@@ -7649,21 +7869,33 @@
 ISNUMBER(SEARCH("RCL*",A16)),"RCL",
 ISNUMBER(SEARCH("SWW*",A16)),"SWW",
 ISNUMBER(SEARCH("MNHV*",A16)),"MNHV")</f>
-        <v>RCL</v>
+        <v>AUHV</v>
       </c>
       <c r="F16" s="1">
-        <v>2.77</v>
+        <v>2.48</v>
       </c>
       <c r="G16" s="1">
-        <v>29.39</v>
+        <v>24.7</v>
+      </c>
+      <c r="H16">
+        <f t="shared" si="0"/>
+        <v>22.22</v>
       </c>
       <c r="I16" s="1">
-        <v>24.01</v>
-      </c>
-    </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.2">
+        <v>21.91</v>
+      </c>
+      <c r="J16">
+        <f t="shared" si="1"/>
+        <v>19.43</v>
+      </c>
+      <c r="K16">
+        <f t="shared" si="2"/>
+        <v>87.443744374437443</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="C17" t="str" cm="1">
         <f t="array" ref="C17">_xlfn.IFS(
@@ -7671,7 +7903,7 @@
 ISNUMBER(SEARCH("III*",A17)),"III",
 ISNUMBER(SEARCH("II*",A17)),"II",
 ISNUMBER(SEARCH("I*",A17)),"I")</f>
-        <v>III</v>
+        <v>I</v>
       </c>
       <c r="D17" cm="1">
         <f t="array" ref="D17">_xlfn.IFS(
@@ -7690,21 +7922,33 @@
 ISNUMBER(SEARCH("RCL*",A17)),"RCL",
 ISNUMBER(SEARCH("SWW*",A17)),"SWW",
 ISNUMBER(SEARCH("MNHV*",A17)),"MNHV")</f>
-        <v>RCL</v>
+        <v>AUHV</v>
       </c>
       <c r="F17" s="1">
-        <v>2.76</v>
+        <v>2.56</v>
       </c>
       <c r="G17" s="1">
-        <v>29.05</v>
+        <v>24.19</v>
+      </c>
+      <c r="H17">
+        <f t="shared" si="0"/>
+        <v>21.630000000000003</v>
       </c>
       <c r="I17" s="1">
-        <v>23.65</v>
-      </c>
-    </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.2">
+        <v>21.52</v>
+      </c>
+      <c r="J17">
+        <f t="shared" si="1"/>
+        <v>18.96</v>
+      </c>
+      <c r="K17">
+        <f t="shared" si="2"/>
+        <v>87.656033287101238</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="C18" t="str" cm="1">
         <f t="array" ref="C18">_xlfn.IFS(
@@ -7712,7 +7956,7 @@
 ISNUMBER(SEARCH("III*",A18)),"III",
 ISNUMBER(SEARCH("II*",A18)),"II",
 ISNUMBER(SEARCH("I*",A18)),"I")</f>
-        <v>III</v>
+        <v>I</v>
       </c>
       <c r="D18" cm="1">
         <f t="array" ref="D18">_xlfn.IFS(
@@ -7731,21 +7975,33 @@
 ISNUMBER(SEARCH("RCL*",A18)),"RCL",
 ISNUMBER(SEARCH("SWW*",A18)),"SWW",
 ISNUMBER(SEARCH("MNHV*",A18)),"MNHV")</f>
-        <v>SWW</v>
+        <v>BWW</v>
       </c>
       <c r="F18" s="1">
         <v>2.7</v>
       </c>
       <c r="G18" s="1">
-        <v>25.75</v>
+        <v>26.08</v>
+      </c>
+      <c r="H18">
+        <f t="shared" si="0"/>
+        <v>23.38</v>
       </c>
       <c r="I18" s="1">
-        <v>21.23</v>
-      </c>
-    </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.2">
+        <v>22.34</v>
+      </c>
+      <c r="J18">
+        <f t="shared" si="1"/>
+        <v>19.64</v>
+      </c>
+      <c r="K18">
+        <f t="shared" si="2"/>
+        <v>84.003421727972622</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="C19" t="str" cm="1">
         <f t="array" ref="C19">_xlfn.IFS(
@@ -7753,7 +8009,7 @@
 ISNUMBER(SEARCH("III*",A19)),"III",
 ISNUMBER(SEARCH("II*",A19)),"II",
 ISNUMBER(SEARCH("I*",A19)),"I")</f>
-        <v>III</v>
+        <v>I</v>
       </c>
       <c r="D19" cm="1">
         <f t="array" ref="D19">_xlfn.IFS(
@@ -7772,21 +8028,33 @@
 ISNUMBER(SEARCH("RCL*",A19)),"RCL",
 ISNUMBER(SEARCH("SWW*",A19)),"SWW",
 ISNUMBER(SEARCH("MNHV*",A19)),"MNHV")</f>
-        <v>SWW</v>
+        <v>BWW</v>
       </c>
       <c r="F19" s="1">
-        <v>2.69</v>
+        <v>2.71</v>
       </c>
       <c r="G19" s="1">
-        <v>26.58</v>
+        <v>25.08</v>
+      </c>
+      <c r="H19">
+        <f t="shared" si="0"/>
+        <v>22.369999999999997</v>
       </c>
       <c r="I19" s="1">
-        <v>21.44</v>
-      </c>
-    </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.2">
+        <v>21.58</v>
+      </c>
+      <c r="J19">
+        <f t="shared" si="1"/>
+        <v>18.869999999999997</v>
+      </c>
+      <c r="K19">
+        <f t="shared" si="2"/>
+        <v>84.354045596781404</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="C20" t="str" cm="1">
         <f t="array" ref="C20">_xlfn.IFS(
@@ -7813,21 +8081,33 @@
 ISNUMBER(SEARCH("RCL*",A20)),"RCL",
 ISNUMBER(SEARCH("SWW*",A20)),"SWW",
 ISNUMBER(SEARCH("MNHV*",A20)),"MNHV")</f>
-        <v>AUHV</v>
+        <v>C1</v>
       </c>
       <c r="F20" s="1">
-        <v>2.48</v>
+        <v>2.71</v>
       </c>
       <c r="G20" s="1">
-        <v>24.7</v>
+        <v>27.19</v>
+      </c>
+      <c r="H20">
+        <f t="shared" si="0"/>
+        <v>24.48</v>
       </c>
       <c r="I20" s="1">
-        <v>21.91</v>
-      </c>
-    </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.2">
+        <v>23.33</v>
+      </c>
+      <c r="J20">
+        <f t="shared" si="1"/>
+        <v>20.619999999999997</v>
+      </c>
+      <c r="K20">
+        <f t="shared" si="2"/>
+        <v>84.232026143790833</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="C21" t="str" cm="1">
         <f t="array" ref="C21">_xlfn.IFS(
@@ -7854,21 +8134,33 @@
 ISNUMBER(SEARCH("RCL*",A21)),"RCL",
 ISNUMBER(SEARCH("SWW*",A21)),"SWW",
 ISNUMBER(SEARCH("MNHV*",A21)),"MNHV")</f>
-        <v>AUHV</v>
+        <v>C1</v>
       </c>
       <c r="F21" s="1">
-        <v>2.56</v>
+        <v>2.71</v>
       </c>
       <c r="G21" s="1">
-        <v>24.19</v>
+        <v>25.88</v>
+      </c>
+      <c r="H21">
+        <f t="shared" si="0"/>
+        <v>23.169999999999998</v>
       </c>
       <c r="I21" s="1">
-        <v>21.52</v>
-      </c>
-    </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.2">
+        <v>22.15</v>
+      </c>
+      <c r="J21">
+        <f t="shared" si="1"/>
+        <v>19.439999999999998</v>
+      </c>
+      <c r="K21">
+        <f t="shared" si="2"/>
+        <v>83.901596892533448</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="C22" t="str" cm="1">
         <f t="array" ref="C22">_xlfn.IFS(
@@ -7895,21 +8187,33 @@
 ISNUMBER(SEARCH("RCL*",A22)),"RCL",
 ISNUMBER(SEARCH("SWW*",A22)),"SWW",
 ISNUMBER(SEARCH("MNHV*",A22)),"MNHV")</f>
-        <v>BWW</v>
+        <v>C2</v>
       </c>
       <c r="F22" s="1">
-        <v>2.7</v>
+        <v>2.71</v>
       </c>
       <c r="G22" s="1">
-        <v>26.08</v>
+        <v>27.45</v>
+      </c>
+      <c r="H22">
+        <f t="shared" si="0"/>
+        <v>24.74</v>
       </c>
       <c r="I22" s="1">
-        <v>22.34</v>
-      </c>
-    </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.2">
+        <v>23.71</v>
+      </c>
+      <c r="J22">
+        <f t="shared" si="1"/>
+        <v>21</v>
+      </c>
+      <c r="K22">
+        <f t="shared" si="2"/>
+        <v>84.882780921584484</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="C23" t="str" cm="1">
         <f t="array" ref="C23">_xlfn.IFS(
@@ -7936,21 +8240,33 @@
 ISNUMBER(SEARCH("RCL*",A23)),"RCL",
 ISNUMBER(SEARCH("SWW*",A23)),"SWW",
 ISNUMBER(SEARCH("MNHV*",A23)),"MNHV")</f>
-        <v>BWW</v>
+        <v>C2</v>
       </c>
       <c r="F23" s="1">
-        <v>2.71</v>
+        <v>2.7</v>
       </c>
       <c r="G23" s="1">
-        <v>25.08</v>
+        <v>24.69</v>
+      </c>
+      <c r="H23">
+        <f t="shared" si="0"/>
+        <v>21.990000000000002</v>
       </c>
       <c r="I23" s="1">
-        <v>21.58</v>
-      </c>
-    </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.2">
+        <v>21.39</v>
+      </c>
+      <c r="J23">
+        <f t="shared" si="1"/>
+        <v>18.690000000000001</v>
+      </c>
+      <c r="K23">
+        <f t="shared" si="2"/>
+        <v>84.993178717598909</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="C24" t="str" cm="1">
         <f t="array" ref="C24">_xlfn.IFS(
@@ -7977,21 +8293,33 @@
 ISNUMBER(SEARCH("RCL*",A24)),"RCL",
 ISNUMBER(SEARCH("SWW*",A24)),"SWW",
 ISNUMBER(SEARCH("MNHV*",A24)),"MNHV")</f>
-        <v>C1</v>
+        <v>MNHV</v>
       </c>
       <c r="F24" s="1">
-        <v>2.71</v>
+        <v>2.52</v>
       </c>
       <c r="G24" s="1">
-        <v>27.19</v>
+        <v>27.06</v>
+      </c>
+      <c r="H24">
+        <f t="shared" si="0"/>
+        <v>24.54</v>
       </c>
       <c r="I24" s="1">
-        <v>23.33</v>
-      </c>
-    </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.2">
+        <v>23.21</v>
+      </c>
+      <c r="J24">
+        <f t="shared" si="1"/>
+        <v>20.69</v>
+      </c>
+      <c r="K24">
+        <f t="shared" si="2"/>
+        <v>84.311328443357795</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="C25" t="str" cm="1">
         <f t="array" ref="C25">_xlfn.IFS(
@@ -8018,21 +8346,33 @@
 ISNUMBER(SEARCH("RCL*",A25)),"RCL",
 ISNUMBER(SEARCH("SWW*",A25)),"SWW",
 ISNUMBER(SEARCH("MNHV*",A25)),"MNHV")</f>
-        <v>C1</v>
+        <v>MNHV</v>
       </c>
       <c r="F25" s="1">
-        <v>2.71</v>
+        <v>2.5099999999999998</v>
       </c>
       <c r="G25" s="1">
-        <v>25.88</v>
+        <v>28.92</v>
+      </c>
+      <c r="H25">
+        <f t="shared" si="0"/>
+        <v>26.410000000000004</v>
       </c>
       <c r="I25" s="1">
-        <v>22.15</v>
-      </c>
-    </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.2">
+        <v>20.63</v>
+      </c>
+      <c r="J25">
+        <f t="shared" si="1"/>
+        <v>18.119999999999997</v>
+      </c>
+      <c r="K25">
+        <f t="shared" si="2"/>
+        <v>68.610374858008313</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="C26" t="str" cm="1">
         <f t="array" ref="C26">_xlfn.IFS(
@@ -8059,21 +8399,33 @@
 ISNUMBER(SEARCH("RCL*",A26)),"RCL",
 ISNUMBER(SEARCH("SWW*",A26)),"SWW",
 ISNUMBER(SEARCH("MNHV*",A26)),"MNHV")</f>
-        <v>C2</v>
+        <v>ORG</v>
       </c>
       <c r="F26" s="1">
-        <v>2.71</v>
+        <v>2.62</v>
       </c>
       <c r="G26" s="1">
-        <v>27.45</v>
+        <v>24.94</v>
+      </c>
+      <c r="H26">
+        <f t="shared" si="0"/>
+        <v>22.32</v>
       </c>
       <c r="I26" s="1">
-        <v>23.71</v>
-      </c>
-    </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.2">
+        <v>22.41</v>
+      </c>
+      <c r="J26">
+        <f t="shared" si="1"/>
+        <v>19.79</v>
+      </c>
+      <c r="K26">
+        <f t="shared" si="2"/>
+        <v>88.664874551971323</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="C27" t="str" cm="1">
         <f t="array" ref="C27">_xlfn.IFS(
@@ -8100,21 +8452,33 @@
 ISNUMBER(SEARCH("RCL*",A27)),"RCL",
 ISNUMBER(SEARCH("SWW*",A27)),"SWW",
 ISNUMBER(SEARCH("MNHV*",A27)),"MNHV")</f>
-        <v>C2</v>
+        <v>ORG</v>
       </c>
       <c r="F27" s="1">
-        <v>2.7</v>
+        <v>2.5499999999999998</v>
       </c>
       <c r="G27" s="1">
-        <v>24.69</v>
+        <v>25.08</v>
+      </c>
+      <c r="H27">
+        <f t="shared" si="0"/>
+        <v>22.529999999999998</v>
       </c>
       <c r="I27" s="1">
-        <v>21.39</v>
-      </c>
-    </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.2">
+        <v>23.06</v>
+      </c>
+      <c r="J27">
+        <f t="shared" si="1"/>
+        <v>20.509999999999998</v>
+      </c>
+      <c r="K27">
+        <f t="shared" si="2"/>
+        <v>91.034176653351082</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="C28" t="str" cm="1">
         <f t="array" ref="C28">_xlfn.IFS(
@@ -8141,21 +8505,33 @@
 ISNUMBER(SEARCH("RCL*",A28)),"RCL",
 ISNUMBER(SEARCH("SWW*",A28)),"SWW",
 ISNUMBER(SEARCH("MNHV*",A28)),"MNHV")</f>
-        <v>MNHV</v>
+        <v>PRY</v>
       </c>
       <c r="F28" s="1">
-        <v>2.52</v>
+        <v>2.58</v>
       </c>
       <c r="G28" s="1">
-        <v>27.06</v>
+        <v>25.39</v>
+      </c>
+      <c r="H28">
+        <f t="shared" si="0"/>
+        <v>22.810000000000002</v>
       </c>
       <c r="I28" s="1">
-        <v>23.21</v>
-      </c>
-    </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.2">
+        <v>22.04</v>
+      </c>
+      <c r="J28">
+        <f t="shared" si="1"/>
+        <v>19.46</v>
+      </c>
+      <c r="K28">
+        <f t="shared" si="2"/>
+        <v>85.313459009206483</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="C29" t="str" cm="1">
         <f t="array" ref="C29">_xlfn.IFS(
@@ -8182,21 +8558,33 @@
 ISNUMBER(SEARCH("RCL*",A29)),"RCL",
 ISNUMBER(SEARCH("SWW*",A29)),"SWW",
 ISNUMBER(SEARCH("MNHV*",A29)),"MNHV")</f>
-        <v>MNHV</v>
+        <v>PRY</v>
       </c>
       <c r="F29" s="1">
-        <v>2.5099999999999998</v>
+        <v>2.63</v>
       </c>
       <c r="G29" s="1">
-        <v>28.92</v>
+        <v>25.39</v>
+      </c>
+      <c r="H29">
+        <f t="shared" si="0"/>
+        <v>22.76</v>
       </c>
       <c r="I29" s="1">
-        <v>20.63</v>
-      </c>
-    </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.2">
+        <v>21.64</v>
+      </c>
+      <c r="J29">
+        <f t="shared" si="1"/>
+        <v>19.010000000000002</v>
+      </c>
+      <c r="K29">
+        <f t="shared" si="2"/>
+        <v>83.523725834797887</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="C30" t="str" cm="1">
         <f t="array" ref="C30">_xlfn.IFS(
@@ -8223,21 +8611,33 @@
 ISNUMBER(SEARCH("RCL*",A30)),"RCL",
 ISNUMBER(SEARCH("SWW*",A30)),"SWW",
 ISNUMBER(SEARCH("MNHV*",A30)),"MNHV")</f>
-        <v>ORG</v>
+        <v>RCL</v>
       </c>
       <c r="F30" s="1">
-        <v>2.62</v>
+        <v>2.68</v>
       </c>
       <c r="G30" s="1">
-        <v>24.94</v>
+        <v>27.59</v>
+      </c>
+      <c r="H30">
+        <f t="shared" si="0"/>
+        <v>24.91</v>
       </c>
       <c r="I30" s="1">
-        <v>22.41</v>
-      </c>
-    </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.2">
+        <v>23.98</v>
+      </c>
+      <c r="J30">
+        <f t="shared" si="1"/>
+        <v>21.3</v>
+      </c>
+      <c r="K30">
+        <f t="shared" si="2"/>
+        <v>85.507828181453235</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="C31" t="str" cm="1">
         <f t="array" ref="C31">_xlfn.IFS(
@@ -8264,21 +8664,33 @@
 ISNUMBER(SEARCH("RCL*",A31)),"RCL",
 ISNUMBER(SEARCH("SWW*",A31)),"SWW",
 ISNUMBER(SEARCH("MNHV*",A31)),"MNHV")</f>
-        <v>ORG</v>
+        <v>RCL</v>
       </c>
       <c r="F31" s="1">
-        <v>2.5499999999999998</v>
+        <v>2.62</v>
       </c>
       <c r="G31" s="1">
-        <v>25.08</v>
+        <v>24.63</v>
+      </c>
+      <c r="H31">
+        <f t="shared" si="0"/>
+        <v>22.009999999999998</v>
       </c>
       <c r="I31" s="1">
-        <v>23.06</v>
-      </c>
-    </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.2">
+        <v>21.41</v>
+      </c>
+      <c r="J31">
+        <f t="shared" si="1"/>
+        <v>18.79</v>
+      </c>
+      <c r="K31">
+        <f t="shared" si="2"/>
+        <v>85.370286233530209</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="C32" t="str" cm="1">
         <f t="array" ref="C32">_xlfn.IFS(
@@ -8305,21 +8717,33 @@
 ISNUMBER(SEARCH("RCL*",A32)),"RCL",
 ISNUMBER(SEARCH("SWW*",A32)),"SWW",
 ISNUMBER(SEARCH("MNHV*",A32)),"MNHV")</f>
-        <v>PRY</v>
+        <v>SWW</v>
       </c>
       <c r="F32" s="1">
-        <v>2.58</v>
+        <v>2.64</v>
       </c>
       <c r="G32" s="1">
-        <v>25.39</v>
+        <v>25.63</v>
+      </c>
+      <c r="H32">
+        <f t="shared" si="0"/>
+        <v>22.99</v>
       </c>
       <c r="I32" s="1">
-        <v>22.04</v>
-      </c>
-    </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.2">
+        <v>22.39</v>
+      </c>
+      <c r="J32">
+        <f t="shared" si="1"/>
+        <v>19.75</v>
+      </c>
+      <c r="K32">
+        <f t="shared" si="2"/>
+        <v>85.906916050456729</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="C33" t="str" cm="1">
         <f t="array" ref="C33">_xlfn.IFS(
@@ -8346,21 +8770,33 @@
 ISNUMBER(SEARCH("RCL*",A33)),"RCL",
 ISNUMBER(SEARCH("SWW*",A33)),"SWW",
 ISNUMBER(SEARCH("MNHV*",A33)),"MNHV")</f>
-        <v>PRY</v>
+        <v>SWW</v>
       </c>
       <c r="F33" s="1">
-        <v>2.63</v>
+        <v>2.62</v>
       </c>
       <c r="G33" s="1">
-        <v>25.39</v>
+        <v>23.9</v>
+      </c>
+      <c r="H33">
+        <f t="shared" si="0"/>
+        <v>21.279999999999998</v>
       </c>
       <c r="I33" s="1">
-        <v>21.64</v>
-      </c>
-    </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.2">
+        <v>20.93</v>
+      </c>
+      <c r="J33">
+        <f t="shared" si="1"/>
+        <v>18.309999999999999</v>
+      </c>
+      <c r="K33">
+        <f t="shared" si="2"/>
+        <v>86.043233082706777</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="C34" t="str" cm="1">
         <f t="array" ref="C34">_xlfn.IFS(
@@ -8368,7 +8804,7 @@
 ISNUMBER(SEARCH("III*",A34)),"III",
 ISNUMBER(SEARCH("II*",A34)),"II",
 ISNUMBER(SEARCH("I*",A34)),"I")</f>
-        <v>I</v>
+        <v>II</v>
       </c>
       <c r="D34" cm="1">
         <f t="array" ref="D34">_xlfn.IFS(
@@ -8387,21 +8823,33 @@
 ISNUMBER(SEARCH("RCL*",A34)),"RCL",
 ISNUMBER(SEARCH("SWW*",A34)),"SWW",
 ISNUMBER(SEARCH("MNHV*",A34)),"MNHV")</f>
-        <v>RCL</v>
+        <v>AUHV</v>
       </c>
       <c r="F34" s="1">
-        <v>2.68</v>
+        <v>2.46</v>
       </c>
       <c r="G34" s="1">
-        <v>27.59</v>
+        <v>25.7</v>
+      </c>
+      <c r="H34">
+        <f t="shared" si="0"/>
+        <v>23.24</v>
       </c>
       <c r="I34" s="1">
-        <v>23.98</v>
-      </c>
-    </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.2">
+        <v>22.28</v>
+      </c>
+      <c r="J34">
+        <f t="shared" si="1"/>
+        <v>19.82</v>
+      </c>
+      <c r="K34">
+        <f t="shared" si="2"/>
+        <v>85.283993115318424</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="C35" t="str" cm="1">
         <f t="array" ref="C35">_xlfn.IFS(
@@ -8409,7 +8857,7 @@
 ISNUMBER(SEARCH("III*",A35)),"III",
 ISNUMBER(SEARCH("II*",A35)),"II",
 ISNUMBER(SEARCH("I*",A35)),"I")</f>
-        <v>I</v>
+        <v>II</v>
       </c>
       <c r="D35" cm="1">
         <f t="array" ref="D35">_xlfn.IFS(
@@ -8428,21 +8876,33 @@
 ISNUMBER(SEARCH("RCL*",A35)),"RCL",
 ISNUMBER(SEARCH("SWW*",A35)),"SWW",
 ISNUMBER(SEARCH("MNHV*",A35)),"MNHV")</f>
-        <v>RCL</v>
+        <v>AUHV</v>
       </c>
       <c r="F35" s="1">
-        <v>2.62</v>
+        <v>2.5099999999999998</v>
       </c>
       <c r="G35" s="1">
-        <v>24.63</v>
+        <v>24.43</v>
+      </c>
+      <c r="H35">
+        <f t="shared" si="0"/>
+        <v>21.92</v>
       </c>
       <c r="I35" s="1">
-        <v>21.41</v>
-      </c>
-    </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.2">
+        <v>20.99</v>
+      </c>
+      <c r="J35">
+        <f t="shared" si="1"/>
+        <v>18.479999999999997</v>
+      </c>
+      <c r="K35">
+        <f t="shared" si="2"/>
+        <v>84.306569343065675</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="C36" t="str" cm="1">
         <f t="array" ref="C36">_xlfn.IFS(
@@ -8450,7 +8910,7 @@
 ISNUMBER(SEARCH("III*",A36)),"III",
 ISNUMBER(SEARCH("II*",A36)),"II",
 ISNUMBER(SEARCH("I*",A36)),"I")</f>
-        <v>I</v>
+        <v>II</v>
       </c>
       <c r="D36" cm="1">
         <f t="array" ref="D36">_xlfn.IFS(
@@ -8469,21 +8929,33 @@
 ISNUMBER(SEARCH("RCL*",A36)),"RCL",
 ISNUMBER(SEARCH("SWW*",A36)),"SWW",
 ISNUMBER(SEARCH("MNHV*",A36)),"MNHV")</f>
-        <v>SWW</v>
+        <v>BWW</v>
       </c>
       <c r="F36" s="1">
-        <v>2.64</v>
+        <v>2.69</v>
       </c>
       <c r="G36" s="1">
-        <v>25.63</v>
+        <v>25.61</v>
+      </c>
+      <c r="H36">
+        <f t="shared" si="0"/>
+        <v>22.919999999999998</v>
       </c>
       <c r="I36" s="1">
-        <v>22.39</v>
-      </c>
-    </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.2">
+        <v>22.28</v>
+      </c>
+      <c r="J36">
+        <f t="shared" si="1"/>
+        <v>19.59</v>
+      </c>
+      <c r="K36">
+        <f t="shared" si="2"/>
+        <v>85.471204188481693</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="C37" t="str" cm="1">
         <f t="array" ref="C37">_xlfn.IFS(
@@ -8491,7 +8963,7 @@
 ISNUMBER(SEARCH("III*",A37)),"III",
 ISNUMBER(SEARCH("II*",A37)),"II",
 ISNUMBER(SEARCH("I*",A37)),"I")</f>
-        <v>I</v>
+        <v>II</v>
       </c>
       <c r="D37" cm="1">
         <f t="array" ref="D37">_xlfn.IFS(
@@ -8510,21 +8982,33 @@
 ISNUMBER(SEARCH("RCL*",A37)),"RCL",
 ISNUMBER(SEARCH("SWW*",A37)),"SWW",
 ISNUMBER(SEARCH("MNHV*",A37)),"MNHV")</f>
-        <v>SWW</v>
+        <v>BWW</v>
       </c>
       <c r="F37" s="1">
-        <v>2.62</v>
+        <v>2.65</v>
       </c>
       <c r="G37" s="1">
-        <v>23.9</v>
+        <v>26.67</v>
+      </c>
+      <c r="H37">
+        <f t="shared" si="0"/>
+        <v>24.020000000000003</v>
       </c>
       <c r="I37" s="1">
-        <v>20.93</v>
-      </c>
-    </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.2">
+        <v>22.96</v>
+      </c>
+      <c r="J37">
+        <f t="shared" si="1"/>
+        <v>20.310000000000002</v>
+      </c>
+      <c r="K37">
+        <f t="shared" si="2"/>
+        <v>84.554537885095755</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>130</v>
+        <v>138</v>
       </c>
       <c r="C38" t="str" cm="1">
         <f t="array" ref="C38">_xlfn.IFS(
@@ -8551,21 +9035,33 @@
 ISNUMBER(SEARCH("RCL*",A38)),"RCL",
 ISNUMBER(SEARCH("SWW*",A38)),"SWW",
 ISNUMBER(SEARCH("MNHV*",A38)),"MNHV")</f>
-        <v>AUHV</v>
+        <v>MNHV</v>
       </c>
       <c r="F38" s="1">
-        <v>2.46</v>
+        <v>2.39</v>
       </c>
       <c r="G38" s="1">
-        <v>25.7</v>
+        <v>29.88</v>
+      </c>
+      <c r="H38">
+        <f t="shared" si="0"/>
+        <v>27.49</v>
       </c>
       <c r="I38" s="1">
-        <v>22.28</v>
-      </c>
-    </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.2">
+        <v>26.74</v>
+      </c>
+      <c r="J38">
+        <f t="shared" si="1"/>
+        <v>24.349999999999998</v>
+      </c>
+      <c r="K38">
+        <f t="shared" si="2"/>
+        <v>88.577664605311028</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>131</v>
+        <v>139</v>
       </c>
       <c r="C39" t="str" cm="1">
         <f t="array" ref="C39">_xlfn.IFS(
@@ -8592,21 +9088,33 @@
 ISNUMBER(SEARCH("RCL*",A39)),"RCL",
 ISNUMBER(SEARCH("SWW*",A39)),"SWW",
 ISNUMBER(SEARCH("MNHV*",A39)),"MNHV")</f>
-        <v>AUHV</v>
+        <v>MNHV</v>
       </c>
       <c r="F39" s="1">
-        <v>2.5099999999999998</v>
+        <v>2.56</v>
       </c>
       <c r="G39" s="1">
-        <v>24.43</v>
+        <v>26.23</v>
+      </c>
+      <c r="H39">
+        <f t="shared" si="0"/>
+        <v>23.67</v>
       </c>
       <c r="I39" s="1">
-        <v>20.99</v>
-      </c>
-    </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.2">
+        <v>23.35</v>
+      </c>
+      <c r="J39">
+        <f t="shared" si="1"/>
+        <v>20.790000000000003</v>
+      </c>
+      <c r="K39">
+        <f t="shared" si="2"/>
+        <v>87.832699619771873</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>132</v>
+        <v>140</v>
       </c>
       <c r="C40" t="str" cm="1">
         <f t="array" ref="C40">_xlfn.IFS(
@@ -8633,21 +9141,33 @@
 ISNUMBER(SEARCH("RCL*",A40)),"RCL",
 ISNUMBER(SEARCH("SWW*",A40)),"SWW",
 ISNUMBER(SEARCH("MNHV*",A40)),"MNHV")</f>
-        <v>BWW</v>
+        <v>ORG</v>
       </c>
       <c r="F40" s="1">
-        <v>2.69</v>
+        <v>2.61</v>
       </c>
       <c r="G40" s="1">
-        <v>25.61</v>
+        <v>27.38</v>
+      </c>
+      <c r="H40">
+        <f t="shared" si="0"/>
+        <v>24.77</v>
       </c>
       <c r="I40" s="1">
-        <v>22.28</v>
-      </c>
-    </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.2">
+        <v>25.15</v>
+      </c>
+      <c r="J40">
+        <f t="shared" si="1"/>
+        <v>22.54</v>
+      </c>
+      <c r="K40">
+        <f t="shared" si="2"/>
+        <v>90.997174000807419</v>
+      </c>
+    </row>
+    <row r="41" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="C41" t="str" cm="1">
         <f t="array" ref="C41">_xlfn.IFS(
@@ -8674,21 +9194,33 @@
 ISNUMBER(SEARCH("RCL*",A41)),"RCL",
 ISNUMBER(SEARCH("SWW*",A41)),"SWW",
 ISNUMBER(SEARCH("MNHV*",A41)),"MNHV")</f>
-        <v>BWW</v>
+        <v>ORG</v>
       </c>
       <c r="F41" s="1">
-        <v>2.65</v>
+        <v>2.59</v>
       </c>
       <c r="G41" s="1">
-        <v>26.67</v>
+        <v>25.45</v>
+      </c>
+      <c r="H41">
+        <f t="shared" si="0"/>
+        <v>22.86</v>
       </c>
       <c r="I41" s="1">
-        <v>22.96</v>
-      </c>
-    </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.2">
+        <v>23.31</v>
+      </c>
+      <c r="J41">
+        <f t="shared" si="1"/>
+        <v>20.72</v>
+      </c>
+      <c r="K41">
+        <f t="shared" si="2"/>
+        <v>90.638670166229218</v>
+      </c>
+    </row>
+    <row r="42" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>134</v>
+        <v>142</v>
       </c>
       <c r="C42" t="str" cm="1">
         <f t="array" ref="C42">_xlfn.IFS(
@@ -8715,12 +9247,33 @@
 ISNUMBER(SEARCH("RCL*",A42)),"RCL",
 ISNUMBER(SEARCH("SWW*",A42)),"SWW",
 ISNUMBER(SEARCH("MNHV*",A42)),"MNHV")</f>
-        <v>C1</v>
-      </c>
-    </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.2">
+        <v>PRY</v>
+      </c>
+      <c r="F42" s="1">
+        <v>2.5499999999999998</v>
+      </c>
+      <c r="G42" s="1">
+        <v>27.19</v>
+      </c>
+      <c r="H42">
+        <f t="shared" si="0"/>
+        <v>24.64</v>
+      </c>
+      <c r="I42" s="1">
+        <v>23.7</v>
+      </c>
+      <c r="J42">
+        <f t="shared" si="1"/>
+        <v>21.15</v>
+      </c>
+      <c r="K42">
+        <f t="shared" si="2"/>
+        <v>85.836038961038952</v>
+      </c>
+    </row>
+    <row r="43" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>135</v>
+        <v>143</v>
       </c>
       <c r="C43" t="str" cm="1">
         <f t="array" ref="C43">_xlfn.IFS(
@@ -8747,12 +9300,33 @@
 ISNUMBER(SEARCH("RCL*",A43)),"RCL",
 ISNUMBER(SEARCH("SWW*",A43)),"SWW",
 ISNUMBER(SEARCH("MNHV*",A43)),"MNHV")</f>
-        <v>C1</v>
-      </c>
-    </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.2">
+        <v>PRY</v>
+      </c>
+      <c r="F43" s="1">
+        <v>2.6</v>
+      </c>
+      <c r="G43" s="1">
+        <v>24.55</v>
+      </c>
+      <c r="H43">
+        <f t="shared" si="0"/>
+        <v>21.95</v>
+      </c>
+      <c r="I43" s="1">
+        <v>21.33</v>
+      </c>
+      <c r="J43">
+        <f t="shared" si="1"/>
+        <v>18.729999999999997</v>
+      </c>
+      <c r="K43">
+        <f t="shared" si="2"/>
+        <v>85.330296127562633</v>
+      </c>
+    </row>
+    <row r="44" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="C44" t="str" cm="1">
         <f t="array" ref="C44">_xlfn.IFS(
@@ -8779,12 +9353,33 @@
 ISNUMBER(SEARCH("RCL*",A44)),"RCL",
 ISNUMBER(SEARCH("SWW*",A44)),"SWW",
 ISNUMBER(SEARCH("MNHV*",A44)),"MNHV")</f>
-        <v>C2</v>
-      </c>
-    </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.2">
+        <v>RCL</v>
+      </c>
+      <c r="F44" s="1">
+        <v>2.61</v>
+      </c>
+      <c r="G44" s="1">
+        <v>24.19</v>
+      </c>
+      <c r="H44">
+        <f t="shared" si="0"/>
+        <v>21.580000000000002</v>
+      </c>
+      <c r="I44" s="1">
+        <v>21.74</v>
+      </c>
+      <c r="J44">
+        <f t="shared" si="1"/>
+        <v>19.13</v>
+      </c>
+      <c r="K44">
+        <f t="shared" si="2"/>
+        <v>88.646895273401284</v>
+      </c>
+    </row>
+    <row r="45" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>137</v>
+        <v>145</v>
       </c>
       <c r="C45" t="str" cm="1">
         <f t="array" ref="C45">_xlfn.IFS(
@@ -8811,12 +9406,33 @@
 ISNUMBER(SEARCH("RCL*",A45)),"RCL",
 ISNUMBER(SEARCH("SWW*",A45)),"SWW",
 ISNUMBER(SEARCH("MNHV*",A45)),"MNHV")</f>
-        <v>C2</v>
-      </c>
-    </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.2">
+        <v>RCL</v>
+      </c>
+      <c r="F45" s="1">
+        <v>2.7</v>
+      </c>
+      <c r="G45" s="1">
+        <v>24.85</v>
+      </c>
+      <c r="H45">
+        <f t="shared" si="0"/>
+        <v>22.150000000000002</v>
+      </c>
+      <c r="I45" s="1">
+        <v>22.37</v>
+      </c>
+      <c r="J45">
+        <f t="shared" si="1"/>
+        <v>19.670000000000002</v>
+      </c>
+      <c r="K45">
+        <f t="shared" si="2"/>
+        <v>88.803611738148973</v>
+      </c>
+    </row>
+    <row r="46" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
       <c r="C46" t="str" cm="1">
         <f t="array" ref="C46">_xlfn.IFS(
@@ -8843,21 +9459,33 @@
 ISNUMBER(SEARCH("RCL*",A46)),"RCL",
 ISNUMBER(SEARCH("SWW*",A46)),"SWW",
 ISNUMBER(SEARCH("MNHV*",A46)),"MNHV")</f>
-        <v>MNHV</v>
+        <v>SWW</v>
       </c>
       <c r="F46" s="1">
-        <v>2.39</v>
+        <v>2.63</v>
       </c>
       <c r="G46" s="1">
-        <v>29.88</v>
+        <v>26.42</v>
+      </c>
+      <c r="H46">
+        <f t="shared" si="0"/>
+        <v>23.790000000000003</v>
       </c>
       <c r="I46" s="1">
-        <v>26.74</v>
-      </c>
-    </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.2">
+        <v>23.42</v>
+      </c>
+      <c r="J46">
+        <f t="shared" si="1"/>
+        <v>20.790000000000003</v>
+      </c>
+      <c r="K46">
+        <f t="shared" si="2"/>
+        <v>87.389659520807058</v>
+      </c>
+    </row>
+    <row r="47" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
-        <v>139</v>
+        <v>147</v>
       </c>
       <c r="C47" t="str" cm="1">
         <f t="array" ref="C47">_xlfn.IFS(
@@ -8884,21 +9512,33 @@
 ISNUMBER(SEARCH("RCL*",A47)),"RCL",
 ISNUMBER(SEARCH("SWW*",A47)),"SWW",
 ISNUMBER(SEARCH("MNHV*",A47)),"MNHV")</f>
-        <v>MNHV</v>
+        <v>SWW</v>
       </c>
       <c r="F47" s="1">
-        <v>2.56</v>
+        <v>2.62</v>
       </c>
       <c r="G47" s="1">
-        <v>26.23</v>
+        <v>25.86</v>
+      </c>
+      <c r="H47">
+        <f t="shared" si="0"/>
+        <v>23.24</v>
       </c>
       <c r="I47" s="1">
-        <v>23.35</v>
-      </c>
-    </row>
-    <row r="48" spans="1:9" x14ac:dyDescent="0.2">
+        <v>22.78</v>
+      </c>
+      <c r="J47">
+        <f t="shared" si="1"/>
+        <v>20.16</v>
+      </c>
+      <c r="K47">
+        <f t="shared" si="2"/>
+        <v>86.746987951807228</v>
+      </c>
+    </row>
+    <row r="48" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
-        <v>140</v>
+        <v>148</v>
       </c>
       <c r="C48" t="str" cm="1">
         <f t="array" ref="C48">_xlfn.IFS(
@@ -8906,7 +9546,7 @@
 ISNUMBER(SEARCH("III*",A48)),"III",
 ISNUMBER(SEARCH("II*",A48)),"II",
 ISNUMBER(SEARCH("I*",A48)),"I")</f>
-        <v>II</v>
+        <v>IV</v>
       </c>
       <c r="D48" cm="1">
         <f t="array" ref="D48">_xlfn.IFS(
@@ -8925,21 +9565,33 @@
 ISNUMBER(SEARCH("RCL*",A48)),"RCL",
 ISNUMBER(SEARCH("SWW*",A48)),"SWW",
 ISNUMBER(SEARCH("MNHV*",A48)),"MNHV")</f>
-        <v>ORG</v>
+        <v>AUHV</v>
       </c>
       <c r="F48" s="1">
-        <v>2.61</v>
+        <v>2.62</v>
       </c>
       <c r="G48" s="1">
-        <v>27.38</v>
+        <v>28.98</v>
+      </c>
+      <c r="H48">
+        <f t="shared" si="0"/>
+        <v>26.36</v>
       </c>
       <c r="I48" s="1">
-        <v>25.15</v>
-      </c>
-    </row>
-    <row r="49" spans="1:9" x14ac:dyDescent="0.2">
+        <v>23.37</v>
+      </c>
+      <c r="J48">
+        <f t="shared" si="1"/>
+        <v>20.75</v>
+      </c>
+      <c r="K48">
+        <f t="shared" si="2"/>
+        <v>78.717754172989387</v>
+      </c>
+    </row>
+    <row r="49" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
-        <v>141</v>
+        <v>149</v>
       </c>
       <c r="C49" t="str" cm="1">
         <f t="array" ref="C49">_xlfn.IFS(
@@ -8947,7 +9599,7 @@
 ISNUMBER(SEARCH("III*",A49)),"III",
 ISNUMBER(SEARCH("II*",A49)),"II",
 ISNUMBER(SEARCH("I*",A49)),"I")</f>
-        <v>II</v>
+        <v>IV</v>
       </c>
       <c r="D49" cm="1">
         <f t="array" ref="D49">_xlfn.IFS(
@@ -8966,21 +9618,33 @@
 ISNUMBER(SEARCH("RCL*",A49)),"RCL",
 ISNUMBER(SEARCH("SWW*",A49)),"SWW",
 ISNUMBER(SEARCH("MNHV*",A49)),"MNHV")</f>
-        <v>ORG</v>
+        <v>AUHV</v>
       </c>
       <c r="F49" s="1">
-        <v>2.59</v>
+        <v>2.5099999999999998</v>
       </c>
       <c r="G49" s="1">
-        <v>25.45</v>
+        <v>27.49</v>
+      </c>
+      <c r="H49">
+        <f t="shared" si="0"/>
+        <v>24.979999999999997</v>
       </c>
       <c r="I49" s="1">
-        <v>23.31</v>
-      </c>
-    </row>
-    <row r="50" spans="1:9" x14ac:dyDescent="0.2">
+        <v>22.22</v>
+      </c>
+      <c r="J49">
+        <f t="shared" si="1"/>
+        <v>19.71</v>
+      </c>
+      <c r="K49">
+        <f t="shared" si="2"/>
+        <v>78.90312249799841</v>
+      </c>
+    </row>
+    <row r="50" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
-        <v>142</v>
+        <v>150</v>
       </c>
       <c r="C50" t="str" cm="1">
         <f t="array" ref="C50">_xlfn.IFS(
@@ -8988,7 +9652,7 @@
 ISNUMBER(SEARCH("III*",A50)),"III",
 ISNUMBER(SEARCH("II*",A50)),"II",
 ISNUMBER(SEARCH("I*",A50)),"I")</f>
-        <v>II</v>
+        <v>IV</v>
       </c>
       <c r="D50" cm="1">
         <f t="array" ref="D50">_xlfn.IFS(
@@ -9007,21 +9671,33 @@
 ISNUMBER(SEARCH("RCL*",A50)),"RCL",
 ISNUMBER(SEARCH("SWW*",A50)),"SWW",
 ISNUMBER(SEARCH("MNHV*",A50)),"MNHV")</f>
-        <v>PRY</v>
+        <v>BWW</v>
       </c>
       <c r="F50" s="1">
-        <v>2.5499999999999998</v>
+        <v>2.62</v>
       </c>
       <c r="G50" s="1">
-        <v>27.19</v>
+        <v>28.28</v>
+      </c>
+      <c r="H50">
+        <f t="shared" si="0"/>
+        <v>25.66</v>
       </c>
       <c r="I50" s="1">
-        <v>23.7</v>
-      </c>
-    </row>
-    <row r="51" spans="1:9" x14ac:dyDescent="0.2">
+        <v>23.34</v>
+      </c>
+      <c r="J50">
+        <f t="shared" si="1"/>
+        <v>20.72</v>
+      </c>
+      <c r="K50">
+        <f t="shared" si="2"/>
+        <v>80.748246297739669</v>
+      </c>
+    </row>
+    <row r="51" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
-        <v>143</v>
+        <v>151</v>
       </c>
       <c r="C51" t="str" cm="1">
         <f t="array" ref="C51">_xlfn.IFS(
@@ -9029,7 +9705,7 @@
 ISNUMBER(SEARCH("III*",A51)),"III",
 ISNUMBER(SEARCH("II*",A51)),"II",
 ISNUMBER(SEARCH("I*",A51)),"I")</f>
-        <v>II</v>
+        <v>IV</v>
       </c>
       <c r="D51" cm="1">
         <f t="array" ref="D51">_xlfn.IFS(
@@ -9048,21 +9724,33 @@
 ISNUMBER(SEARCH("RCL*",A51)),"RCL",
 ISNUMBER(SEARCH("SWW*",A51)),"SWW",
 ISNUMBER(SEARCH("MNHV*",A51)),"MNHV")</f>
-        <v>PRY</v>
+        <v>BWW</v>
       </c>
       <c r="F51" s="1">
-        <v>2.6</v>
+        <v>2.61</v>
       </c>
       <c r="G51" s="1">
-        <v>24.55</v>
+        <v>25.96</v>
+      </c>
+      <c r="H51">
+        <f t="shared" si="0"/>
+        <v>23.35</v>
       </c>
       <c r="I51" s="1">
-        <v>21.33</v>
-      </c>
-    </row>
-    <row r="52" spans="1:9" x14ac:dyDescent="0.2">
+        <v>22.44</v>
+      </c>
+      <c r="J51">
+        <f t="shared" si="1"/>
+        <v>19.830000000000002</v>
+      </c>
+      <c r="K51">
+        <f t="shared" si="2"/>
+        <v>84.925053533190578</v>
+      </c>
+    </row>
+    <row r="52" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
-        <v>144</v>
+        <v>156</v>
       </c>
       <c r="C52" t="str" cm="1">
         <f t="array" ref="C52">_xlfn.IFS(
@@ -9070,7 +9758,7 @@
 ISNUMBER(SEARCH("III*",A52)),"III",
 ISNUMBER(SEARCH("II*",A52)),"II",
 ISNUMBER(SEARCH("I*",A52)),"I")</f>
-        <v>II</v>
+        <v>IV</v>
       </c>
       <c r="D52" cm="1">
         <f t="array" ref="D52">_xlfn.IFS(
@@ -9089,21 +9777,33 @@
 ISNUMBER(SEARCH("RCL*",A52)),"RCL",
 ISNUMBER(SEARCH("SWW*",A52)),"SWW",
 ISNUMBER(SEARCH("MNHV*",A52)),"MNHV")</f>
-        <v>RCL</v>
+        <v>MNHV</v>
       </c>
       <c r="F52" s="1">
-        <v>2.61</v>
+        <v>2.65</v>
       </c>
       <c r="G52" s="1">
-        <v>24.19</v>
+        <v>27.16</v>
+      </c>
+      <c r="H52">
+        <f t="shared" si="0"/>
+        <v>24.51</v>
       </c>
       <c r="I52" s="1">
-        <v>21.74</v>
-      </c>
-    </row>
-    <row r="53" spans="1:9" x14ac:dyDescent="0.2">
+        <v>22.27</v>
+      </c>
+      <c r="J52">
+        <f t="shared" si="1"/>
+        <v>19.62</v>
+      </c>
+      <c r="K52">
+        <f t="shared" si="2"/>
+        <v>80.048959608323131</v>
+      </c>
+    </row>
+    <row r="53" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
-        <v>145</v>
+        <v>157</v>
       </c>
       <c r="C53" t="str" cm="1">
         <f t="array" ref="C53">_xlfn.IFS(
@@ -9111,7 +9811,7 @@
 ISNUMBER(SEARCH("III*",A53)),"III",
 ISNUMBER(SEARCH("II*",A53)),"II",
 ISNUMBER(SEARCH("I*",A53)),"I")</f>
-        <v>II</v>
+        <v>IV</v>
       </c>
       <c r="D53" cm="1">
         <f t="array" ref="D53">_xlfn.IFS(
@@ -9130,21 +9830,33 @@
 ISNUMBER(SEARCH("RCL*",A53)),"RCL",
 ISNUMBER(SEARCH("SWW*",A53)),"SWW",
 ISNUMBER(SEARCH("MNHV*",A53)),"MNHV")</f>
-        <v>RCL</v>
+        <v>MNHV</v>
       </c>
       <c r="F53" s="1">
-        <v>2.7</v>
+        <v>2.59</v>
       </c>
       <c r="G53" s="1">
-        <v>24.85</v>
+        <v>25.49</v>
+      </c>
+      <c r="H53">
+        <f t="shared" si="0"/>
+        <v>22.9</v>
       </c>
       <c r="I53" s="1">
-        <v>22.37</v>
-      </c>
-    </row>
-    <row r="54" spans="1:9" x14ac:dyDescent="0.2">
+        <v>21.09</v>
+      </c>
+      <c r="J53">
+        <f t="shared" si="1"/>
+        <v>18.5</v>
+      </c>
+      <c r="K53">
+        <f t="shared" si="2"/>
+        <v>80.786026200873366</v>
+      </c>
+    </row>
+    <row r="54" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
-        <v>146</v>
+        <v>158</v>
       </c>
       <c r="C54" t="str" cm="1">
         <f t="array" ref="C54">_xlfn.IFS(
@@ -9152,7 +9864,7 @@
 ISNUMBER(SEARCH("III*",A54)),"III",
 ISNUMBER(SEARCH("II*",A54)),"II",
 ISNUMBER(SEARCH("I*",A54)),"I")</f>
-        <v>II</v>
+        <v>IV</v>
       </c>
       <c r="D54" cm="1">
         <f t="array" ref="D54">_xlfn.IFS(
@@ -9171,21 +9883,33 @@
 ISNUMBER(SEARCH("RCL*",A54)),"RCL",
 ISNUMBER(SEARCH("SWW*",A54)),"SWW",
 ISNUMBER(SEARCH("MNHV*",A54)),"MNHV")</f>
-        <v>SWW</v>
+        <v>ORG</v>
       </c>
       <c r="F54" s="1">
-        <v>2.63</v>
+        <v>2.64</v>
       </c>
       <c r="G54" s="1">
-        <v>26.42</v>
+        <v>25.79</v>
+      </c>
+      <c r="H54">
+        <f t="shared" si="0"/>
+        <v>23.15</v>
       </c>
       <c r="I54" s="1">
-        <v>23.42</v>
-      </c>
-    </row>
-    <row r="55" spans="1:9" x14ac:dyDescent="0.2">
+        <v>21.17</v>
+      </c>
+      <c r="J54">
+        <f t="shared" si="1"/>
+        <v>18.53</v>
+      </c>
+      <c r="K54">
+        <f t="shared" si="2"/>
+        <v>80.043196544276469</v>
+      </c>
+    </row>
+    <row r="55" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
-        <v>147</v>
+        <v>159</v>
       </c>
       <c r="C55" t="str" cm="1">
         <f t="array" ref="C55">_xlfn.IFS(
@@ -9193,7 +9917,7 @@
 ISNUMBER(SEARCH("III*",A55)),"III",
 ISNUMBER(SEARCH("II*",A55)),"II",
 ISNUMBER(SEARCH("I*",A55)),"I")</f>
-        <v>II</v>
+        <v>IV</v>
       </c>
       <c r="D55" cm="1">
         <f t="array" ref="D55">_xlfn.IFS(
@@ -9212,21 +9936,33 @@
 ISNUMBER(SEARCH("RCL*",A55)),"RCL",
 ISNUMBER(SEARCH("SWW*",A55)),"SWW",
 ISNUMBER(SEARCH("MNHV*",A55)),"MNHV")</f>
-        <v>SWW</v>
+        <v>ORG</v>
       </c>
       <c r="F55" s="1">
-        <v>2.62</v>
+        <v>2.69</v>
       </c>
       <c r="G55" s="1">
-        <v>25.86</v>
+        <v>26.93</v>
+      </c>
+      <c r="H55">
+        <f t="shared" ref="H55:H61" si="3">G55-F55</f>
+        <v>24.24</v>
       </c>
       <c r="I55" s="1">
-        <v>22.78</v>
-      </c>
-    </row>
-    <row r="56" spans="1:9" x14ac:dyDescent="0.2">
+        <v>22.59</v>
+      </c>
+      <c r="J55">
+        <f t="shared" ref="J55:J61" si="4">I55-F55</f>
+        <v>19.899999999999999</v>
+      </c>
+      <c r="K55">
+        <f t="shared" ref="K55:K61" si="5">J55/H55*100</f>
+        <v>82.095709570957098</v>
+      </c>
+    </row>
+    <row r="56" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
-        <v>148</v>
+        <v>160</v>
       </c>
       <c r="C56" t="str" cm="1">
         <f t="array" ref="C56">_xlfn.IFS(
@@ -9253,21 +9989,33 @@
 ISNUMBER(SEARCH("RCL*",A56)),"RCL",
 ISNUMBER(SEARCH("SWW*",A56)),"SWW",
 ISNUMBER(SEARCH("MNHV*",A56)),"MNHV")</f>
-        <v>AUHV</v>
+        <v>PRY</v>
       </c>
       <c r="F56" s="1">
-        <v>2.62</v>
+        <v>2.67</v>
       </c>
       <c r="G56" s="1">
-        <v>28.98</v>
+        <v>27.33</v>
+      </c>
+      <c r="H56">
+        <f t="shared" si="3"/>
+        <v>24.659999999999997</v>
       </c>
       <c r="I56" s="1">
-        <v>23.37</v>
-      </c>
-    </row>
-    <row r="57" spans="1:9" x14ac:dyDescent="0.2">
+        <v>22.13</v>
+      </c>
+      <c r="J56">
+        <f t="shared" si="4"/>
+        <v>19.46</v>
+      </c>
+      <c r="K56">
+        <f t="shared" si="5"/>
+        <v>78.913219789132214</v>
+      </c>
+    </row>
+    <row r="57" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
-        <v>149</v>
+        <v>161</v>
       </c>
       <c r="C57" t="str" cm="1">
         <f t="array" ref="C57">_xlfn.IFS(
@@ -9294,21 +10042,33 @@
 ISNUMBER(SEARCH("RCL*",A57)),"RCL",
 ISNUMBER(SEARCH("SWW*",A57)),"SWW",
 ISNUMBER(SEARCH("MNHV*",A57)),"MNHV")</f>
-        <v>AUHV</v>
+        <v>PRY</v>
       </c>
       <c r="F57" s="1">
-        <v>2.5099999999999998</v>
+        <v>2.69</v>
       </c>
       <c r="G57" s="1">
-        <v>27.49</v>
+        <v>28.98</v>
+      </c>
+      <c r="H57">
+        <f t="shared" si="3"/>
+        <v>26.29</v>
       </c>
       <c r="I57" s="1">
-        <v>22.22</v>
-      </c>
-    </row>
-    <row r="58" spans="1:9" x14ac:dyDescent="0.2">
+        <v>24.12</v>
+      </c>
+      <c r="J57">
+        <f t="shared" si="4"/>
+        <v>21.43</v>
+      </c>
+      <c r="K57">
+        <f t="shared" si="5"/>
+        <v>81.513883605933813</v>
+      </c>
+    </row>
+    <row r="58" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
-        <v>150</v>
+        <v>162</v>
       </c>
       <c r="C58" t="str" cm="1">
         <f t="array" ref="C58">_xlfn.IFS(
@@ -9335,21 +10095,33 @@
 ISNUMBER(SEARCH("RCL*",A58)),"RCL",
 ISNUMBER(SEARCH("SWW*",A58)),"SWW",
 ISNUMBER(SEARCH("MNHV*",A58)),"MNHV")</f>
-        <v>BWW</v>
+        <v>RCL</v>
       </c>
       <c r="F58" s="1">
-        <v>2.62</v>
+        <v>2.73</v>
       </c>
       <c r="G58" s="1">
-        <v>28.28</v>
+        <v>29.89</v>
+      </c>
+      <c r="H58">
+        <f t="shared" si="3"/>
+        <v>27.16</v>
       </c>
       <c r="I58" s="1">
-        <v>23.34</v>
-      </c>
-    </row>
-    <row r="59" spans="1:9" x14ac:dyDescent="0.2">
+        <v>25.04</v>
+      </c>
+      <c r="J58">
+        <f t="shared" si="4"/>
+        <v>22.31</v>
+      </c>
+      <c r="K58">
+        <f t="shared" si="5"/>
+        <v>82.142857142857139</v>
+      </c>
+    </row>
+    <row r="59" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
-        <v>151</v>
+        <v>163</v>
       </c>
       <c r="C59" t="str" cm="1">
         <f t="array" ref="C59">_xlfn.IFS(
@@ -9376,21 +10148,33 @@
 ISNUMBER(SEARCH("RCL*",A59)),"RCL",
 ISNUMBER(SEARCH("SWW*",A59)),"SWW",
 ISNUMBER(SEARCH("MNHV*",A59)),"MNHV")</f>
-        <v>BWW</v>
+        <v>RCL</v>
       </c>
       <c r="F59" s="1">
-        <v>2.61</v>
+        <v>2.73</v>
       </c>
       <c r="G59" s="1">
-        <v>25.96</v>
+        <v>29.34</v>
+      </c>
+      <c r="H59">
+        <f t="shared" si="3"/>
+        <v>26.61</v>
       </c>
       <c r="I59" s="1">
-        <v>22.44</v>
-      </c>
-    </row>
-    <row r="60" spans="1:9" x14ac:dyDescent="0.2">
+        <v>24.59</v>
+      </c>
+      <c r="J59">
+        <f t="shared" si="4"/>
+        <v>21.86</v>
+      </c>
+      <c r="K59">
+        <f t="shared" si="5"/>
+        <v>82.14956783164223</v>
+      </c>
+    </row>
+    <row r="60" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
-        <v>152</v>
+        <v>164</v>
       </c>
       <c r="C60" t="str" cm="1">
         <f t="array" ref="C60">_xlfn.IFS(
@@ -9417,12 +10201,33 @@
 ISNUMBER(SEARCH("RCL*",A60)),"RCL",
 ISNUMBER(SEARCH("SWW*",A60)),"SWW",
 ISNUMBER(SEARCH("MNHV*",A60)),"MNHV")</f>
-        <v>C1</v>
-      </c>
-    </row>
-    <row r="61" spans="1:9" x14ac:dyDescent="0.2">
+        <v>SWW</v>
+      </c>
+      <c r="F60" s="1">
+        <v>2.75</v>
+      </c>
+      <c r="G60" s="1">
+        <v>28.72</v>
+      </c>
+      <c r="H60">
+        <f t="shared" si="3"/>
+        <v>25.97</v>
+      </c>
+      <c r="I60" s="1">
+        <v>23.47</v>
+      </c>
+      <c r="J60">
+        <f t="shared" si="4"/>
+        <v>20.72</v>
+      </c>
+      <c r="K60">
+        <f t="shared" si="5"/>
+        <v>79.784366576819409</v>
+      </c>
+    </row>
+    <row r="61" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
-        <v>153</v>
+        <v>165</v>
       </c>
       <c r="C61" t="str" cm="1">
         <f t="array" ref="C61">_xlfn.IFS(
@@ -9449,485 +10254,75 @@
 ISNUMBER(SEARCH("RCL*",A61)),"RCL",
 ISNUMBER(SEARCH("SWW*",A61)),"SWW",
 ISNUMBER(SEARCH("MNHV*",A61)),"MNHV")</f>
-        <v>C1</v>
-      </c>
-    </row>
-    <row r="62" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A62" t="s">
-        <v>154</v>
-      </c>
-      <c r="C62" t="str" cm="1">
-        <f t="array" ref="C62">_xlfn.IFS(
-ISNUMBER(SEARCH("IV*",A62)),"IV",
-ISNUMBER(SEARCH("III*",A62)),"III",
-ISNUMBER(SEARCH("II*",A62)),"II",
-ISNUMBER(SEARCH("I*",A62)),"I")</f>
-        <v>IV</v>
-      </c>
-      <c r="D62" cm="1">
-        <f t="array" ref="D62">_xlfn.IFS(
-ISNUMBER(SEARCH("-1*",A62)),1,
-ISNUMBER(SEARCH("-2*",A62)),2)</f>
-        <v>1</v>
-      </c>
-      <c r="E62" t="str" cm="1">
-        <f t="array" ref="E62">_xlfn.IFS(
-ISNUMBER(SEARCH("AUHV*",A62)),"AUHV",
-ISNUMBER(SEARCH("BWW*",A62)),"BWW",
-ISNUMBER(SEARCH("C1*",A62)),"C1",
-ISNUMBER(SEARCH("C2*",A62)),"C2",
-ISNUMBER(SEARCH("ORG*",A62)),"ORG",
-ISNUMBER(SEARCH("PRY*",A62)),"PRY",
-ISNUMBER(SEARCH("RCL*",A62)),"RCL",
-ISNUMBER(SEARCH("SWW*",A62)),"SWW",
-ISNUMBER(SEARCH("MNHV*",A62)),"MNHV")</f>
-        <v>C2</v>
-      </c>
-    </row>
-    <row r="63" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A63" t="s">
-        <v>155</v>
-      </c>
-      <c r="C63" t="str" cm="1">
-        <f t="array" ref="C63">_xlfn.IFS(
-ISNUMBER(SEARCH("IV*",A63)),"IV",
-ISNUMBER(SEARCH("III*",A63)),"III",
-ISNUMBER(SEARCH("II*",A63)),"II",
-ISNUMBER(SEARCH("I*",A63)),"I")</f>
-        <v>IV</v>
-      </c>
-      <c r="D63" cm="1">
-        <f t="array" ref="D63">_xlfn.IFS(
-ISNUMBER(SEARCH("-1*",A63)),1,
-ISNUMBER(SEARCH("-2*",A63)),2)</f>
-        <v>2</v>
-      </c>
-      <c r="E63" t="str" cm="1">
-        <f t="array" ref="E63">_xlfn.IFS(
-ISNUMBER(SEARCH("AUHV*",A63)),"AUHV",
-ISNUMBER(SEARCH("BWW*",A63)),"BWW",
-ISNUMBER(SEARCH("C1*",A63)),"C1",
-ISNUMBER(SEARCH("C2*",A63)),"C2",
-ISNUMBER(SEARCH("ORG*",A63)),"ORG",
-ISNUMBER(SEARCH("PRY*",A63)),"PRY",
-ISNUMBER(SEARCH("RCL*",A63)),"RCL",
-ISNUMBER(SEARCH("SWW*",A63)),"SWW",
-ISNUMBER(SEARCH("MNHV*",A63)),"MNHV")</f>
-        <v>C2</v>
-      </c>
-    </row>
-    <row r="64" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A64" t="s">
-        <v>156</v>
-      </c>
-      <c r="C64" t="str" cm="1">
-        <f t="array" ref="C64">_xlfn.IFS(
-ISNUMBER(SEARCH("IV*",A64)),"IV",
-ISNUMBER(SEARCH("III*",A64)),"III",
-ISNUMBER(SEARCH("II*",A64)),"II",
-ISNUMBER(SEARCH("I*",A64)),"I")</f>
-        <v>IV</v>
-      </c>
-      <c r="D64" cm="1">
-        <f t="array" ref="D64">_xlfn.IFS(
-ISNUMBER(SEARCH("-1*",A64)),1,
-ISNUMBER(SEARCH("-2*",A64)),2)</f>
-        <v>1</v>
-      </c>
-      <c r="E64" t="str" cm="1">
-        <f t="array" ref="E64">_xlfn.IFS(
-ISNUMBER(SEARCH("AUHV*",A64)),"AUHV",
-ISNUMBER(SEARCH("BWW*",A64)),"BWW",
-ISNUMBER(SEARCH("C1*",A64)),"C1",
-ISNUMBER(SEARCH("C2*",A64)),"C2",
-ISNUMBER(SEARCH("ORG*",A64)),"ORG",
-ISNUMBER(SEARCH("PRY*",A64)),"PRY",
-ISNUMBER(SEARCH("RCL*",A64)),"RCL",
-ISNUMBER(SEARCH("SWW*",A64)),"SWW",
-ISNUMBER(SEARCH("MNHV*",A64)),"MNHV")</f>
-        <v>MNHV</v>
-      </c>
-      <c r="F64" s="1">
-        <v>2.65</v>
-      </c>
-      <c r="G64" s="1">
-        <v>27.16</v>
-      </c>
-      <c r="I64" s="1">
-        <v>22.27</v>
-      </c>
-    </row>
-    <row r="65" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A65" t="s">
-        <v>157</v>
-      </c>
-      <c r="C65" t="str" cm="1">
-        <f t="array" ref="C65">_xlfn.IFS(
-ISNUMBER(SEARCH("IV*",A65)),"IV",
-ISNUMBER(SEARCH("III*",A65)),"III",
-ISNUMBER(SEARCH("II*",A65)),"II",
-ISNUMBER(SEARCH("I*",A65)),"I")</f>
-        <v>IV</v>
-      </c>
-      <c r="D65" cm="1">
-        <f t="array" ref="D65">_xlfn.IFS(
-ISNUMBER(SEARCH("-1*",A65)),1,
-ISNUMBER(SEARCH("-2*",A65)),2)</f>
-        <v>2</v>
-      </c>
-      <c r="E65" t="str" cm="1">
-        <f t="array" ref="E65">_xlfn.IFS(
-ISNUMBER(SEARCH("AUHV*",A65)),"AUHV",
-ISNUMBER(SEARCH("BWW*",A65)),"BWW",
-ISNUMBER(SEARCH("C1*",A65)),"C1",
-ISNUMBER(SEARCH("C2*",A65)),"C2",
-ISNUMBER(SEARCH("ORG*",A65)),"ORG",
-ISNUMBER(SEARCH("PRY*",A65)),"PRY",
-ISNUMBER(SEARCH("RCL*",A65)),"RCL",
-ISNUMBER(SEARCH("SWW*",A65)),"SWW",
-ISNUMBER(SEARCH("MNHV*",A65)),"MNHV")</f>
-        <v>MNHV</v>
-      </c>
-      <c r="F65" s="1">
-        <v>2.59</v>
-      </c>
-      <c r="G65" s="1">
-        <v>25.49</v>
-      </c>
-      <c r="I65" s="1">
-        <v>21.09</v>
-      </c>
-    </row>
-    <row r="66" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A66" t="s">
-        <v>158</v>
-      </c>
-      <c r="C66" t="str" cm="1">
-        <f t="array" ref="C66">_xlfn.IFS(
-ISNUMBER(SEARCH("IV*",A66)),"IV",
-ISNUMBER(SEARCH("III*",A66)),"III",
-ISNUMBER(SEARCH("II*",A66)),"II",
-ISNUMBER(SEARCH("I*",A66)),"I")</f>
-        <v>IV</v>
-      </c>
-      <c r="D66" cm="1">
-        <f t="array" ref="D66">_xlfn.IFS(
-ISNUMBER(SEARCH("-1*",A66)),1,
-ISNUMBER(SEARCH("-2*",A66)),2)</f>
-        <v>1</v>
-      </c>
-      <c r="E66" t="str" cm="1">
-        <f t="array" ref="E66">_xlfn.IFS(
-ISNUMBER(SEARCH("AUHV*",A66)),"AUHV",
-ISNUMBER(SEARCH("BWW*",A66)),"BWW",
-ISNUMBER(SEARCH("C1*",A66)),"C1",
-ISNUMBER(SEARCH("C2*",A66)),"C2",
-ISNUMBER(SEARCH("ORG*",A66)),"ORG",
-ISNUMBER(SEARCH("PRY*",A66)),"PRY",
-ISNUMBER(SEARCH("RCL*",A66)),"RCL",
-ISNUMBER(SEARCH("SWW*",A66)),"SWW",
-ISNUMBER(SEARCH("MNHV*",A66)),"MNHV")</f>
-        <v>ORG</v>
-      </c>
-      <c r="F66" s="1">
-        <v>2.64</v>
-      </c>
-      <c r="G66" s="1">
-        <v>25.79</v>
-      </c>
-      <c r="I66" s="1">
-        <v>21.17</v>
-      </c>
-    </row>
-    <row r="67" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A67" t="s">
-        <v>159</v>
-      </c>
-      <c r="C67" t="str" cm="1">
-        <f t="array" ref="C67">_xlfn.IFS(
-ISNUMBER(SEARCH("IV*",A67)),"IV",
-ISNUMBER(SEARCH("III*",A67)),"III",
-ISNUMBER(SEARCH("II*",A67)),"II",
-ISNUMBER(SEARCH("I*",A67)),"I")</f>
-        <v>IV</v>
-      </c>
-      <c r="D67" cm="1">
-        <f t="array" ref="D67">_xlfn.IFS(
-ISNUMBER(SEARCH("-1*",A67)),1,
-ISNUMBER(SEARCH("-2*",A67)),2)</f>
-        <v>2</v>
-      </c>
-      <c r="E67" t="str" cm="1">
-        <f t="array" ref="E67">_xlfn.IFS(
-ISNUMBER(SEARCH("AUHV*",A67)),"AUHV",
-ISNUMBER(SEARCH("BWW*",A67)),"BWW",
-ISNUMBER(SEARCH("C1*",A67)),"C1",
-ISNUMBER(SEARCH("C2*",A67)),"C2",
-ISNUMBER(SEARCH("ORG*",A67)),"ORG",
-ISNUMBER(SEARCH("PRY*",A67)),"PRY",
-ISNUMBER(SEARCH("RCL*",A67)),"RCL",
-ISNUMBER(SEARCH("SWW*",A67)),"SWW",
-ISNUMBER(SEARCH("MNHV*",A67)),"MNHV")</f>
-        <v>ORG</v>
-      </c>
-      <c r="F67" s="1">
-        <v>2.69</v>
-      </c>
-      <c r="G67" s="1">
-        <v>26.93</v>
-      </c>
-      <c r="I67" s="1">
-        <v>22.59</v>
-      </c>
-    </row>
-    <row r="68" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A68" t="s">
-        <v>160</v>
-      </c>
-      <c r="C68" t="str" cm="1">
-        <f t="array" ref="C68">_xlfn.IFS(
-ISNUMBER(SEARCH("IV*",A68)),"IV",
-ISNUMBER(SEARCH("III*",A68)),"III",
-ISNUMBER(SEARCH("II*",A68)),"II",
-ISNUMBER(SEARCH("I*",A68)),"I")</f>
-        <v>IV</v>
-      </c>
-      <c r="D68" cm="1">
-        <f t="array" ref="D68">_xlfn.IFS(
-ISNUMBER(SEARCH("-1*",A68)),1,
-ISNUMBER(SEARCH("-2*",A68)),2)</f>
-        <v>1</v>
-      </c>
-      <c r="E68" t="str" cm="1">
-        <f t="array" ref="E68">_xlfn.IFS(
-ISNUMBER(SEARCH("AUHV*",A68)),"AUHV",
-ISNUMBER(SEARCH("BWW*",A68)),"BWW",
-ISNUMBER(SEARCH("C1*",A68)),"C1",
-ISNUMBER(SEARCH("C2*",A68)),"C2",
-ISNUMBER(SEARCH("ORG*",A68)),"ORG",
-ISNUMBER(SEARCH("PRY*",A68)),"PRY",
-ISNUMBER(SEARCH("RCL*",A68)),"RCL",
-ISNUMBER(SEARCH("SWW*",A68)),"SWW",
-ISNUMBER(SEARCH("MNHV*",A68)),"MNHV")</f>
-        <v>PRY</v>
-      </c>
-      <c r="F68" s="1">
-        <v>2.67</v>
-      </c>
-      <c r="G68" s="1">
-        <v>27.33</v>
-      </c>
-      <c r="I68" s="1">
-        <v>22.13</v>
-      </c>
-    </row>
-    <row r="69" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A69" t="s">
-        <v>161</v>
-      </c>
-      <c r="C69" t="str" cm="1">
-        <f t="array" ref="C69">_xlfn.IFS(
-ISNUMBER(SEARCH("IV*",A69)),"IV",
-ISNUMBER(SEARCH("III*",A69)),"III",
-ISNUMBER(SEARCH("II*",A69)),"II",
-ISNUMBER(SEARCH("I*",A69)),"I")</f>
-        <v>IV</v>
-      </c>
-      <c r="D69" cm="1">
-        <f t="array" ref="D69">_xlfn.IFS(
-ISNUMBER(SEARCH("-1*",A69)),1,
-ISNUMBER(SEARCH("-2*",A69)),2)</f>
-        <v>2</v>
-      </c>
-      <c r="E69" t="str" cm="1">
-        <f t="array" ref="E69">_xlfn.IFS(
-ISNUMBER(SEARCH("AUHV*",A69)),"AUHV",
-ISNUMBER(SEARCH("BWW*",A69)),"BWW",
-ISNUMBER(SEARCH("C1*",A69)),"C1",
-ISNUMBER(SEARCH("C2*",A69)),"C2",
-ISNUMBER(SEARCH("ORG*",A69)),"ORG",
-ISNUMBER(SEARCH("PRY*",A69)),"PRY",
-ISNUMBER(SEARCH("RCL*",A69)),"RCL",
-ISNUMBER(SEARCH("SWW*",A69)),"SWW",
-ISNUMBER(SEARCH("MNHV*",A69)),"MNHV")</f>
-        <v>PRY</v>
-      </c>
-      <c r="F69" s="1">
-        <v>2.69</v>
-      </c>
-      <c r="G69" s="1">
-        <v>28.98</v>
-      </c>
-      <c r="I69" s="1">
-        <v>24.12</v>
-      </c>
-    </row>
-    <row r="70" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A70" t="s">
-        <v>162</v>
-      </c>
-      <c r="C70" t="str" cm="1">
-        <f t="array" ref="C70">_xlfn.IFS(
-ISNUMBER(SEARCH("IV*",A70)),"IV",
-ISNUMBER(SEARCH("III*",A70)),"III",
-ISNUMBER(SEARCH("II*",A70)),"II",
-ISNUMBER(SEARCH("I*",A70)),"I")</f>
-        <v>IV</v>
-      </c>
-      <c r="D70" cm="1">
-        <f t="array" ref="D70">_xlfn.IFS(
-ISNUMBER(SEARCH("-1*",A70)),1,
-ISNUMBER(SEARCH("-2*",A70)),2)</f>
-        <v>1</v>
-      </c>
-      <c r="E70" t="str" cm="1">
-        <f t="array" ref="E70">_xlfn.IFS(
-ISNUMBER(SEARCH("AUHV*",A70)),"AUHV",
-ISNUMBER(SEARCH("BWW*",A70)),"BWW",
-ISNUMBER(SEARCH("C1*",A70)),"C1",
-ISNUMBER(SEARCH("C2*",A70)),"C2",
-ISNUMBER(SEARCH("ORG*",A70)),"ORG",
-ISNUMBER(SEARCH("PRY*",A70)),"PRY",
-ISNUMBER(SEARCH("RCL*",A70)),"RCL",
-ISNUMBER(SEARCH("SWW*",A70)),"SWW",
-ISNUMBER(SEARCH("MNHV*",A70)),"MNHV")</f>
-        <v>RCL</v>
-      </c>
-      <c r="F70" s="1">
+        <v>SWW</v>
+      </c>
+      <c r="F61" s="1">
         <v>2.73</v>
       </c>
-      <c r="G70" s="1">
-        <v>29.89</v>
-      </c>
-      <c r="I70" s="1">
-        <v>25.04</v>
-      </c>
-    </row>
-    <row r="71" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A71" t="s">
-        <v>163</v>
-      </c>
-      <c r="C71" t="str" cm="1">
-        <f t="array" ref="C71">_xlfn.IFS(
-ISNUMBER(SEARCH("IV*",A71)),"IV",
-ISNUMBER(SEARCH("III*",A71)),"III",
-ISNUMBER(SEARCH("II*",A71)),"II",
-ISNUMBER(SEARCH("I*",A71)),"I")</f>
-        <v>IV</v>
-      </c>
-      <c r="D71" cm="1">
-        <f t="array" ref="D71">_xlfn.IFS(
-ISNUMBER(SEARCH("-1*",A71)),1,
-ISNUMBER(SEARCH("-2*",A71)),2)</f>
-        <v>2</v>
-      </c>
-      <c r="E71" t="str" cm="1">
-        <f t="array" ref="E71">_xlfn.IFS(
-ISNUMBER(SEARCH("AUHV*",A71)),"AUHV",
-ISNUMBER(SEARCH("BWW*",A71)),"BWW",
-ISNUMBER(SEARCH("C1*",A71)),"C1",
-ISNUMBER(SEARCH("C2*",A71)),"C2",
-ISNUMBER(SEARCH("ORG*",A71)),"ORG",
-ISNUMBER(SEARCH("PRY*",A71)),"PRY",
-ISNUMBER(SEARCH("RCL*",A71)),"RCL",
-ISNUMBER(SEARCH("SWW*",A71)),"SWW",
-ISNUMBER(SEARCH("MNHV*",A71)),"MNHV")</f>
-        <v>RCL</v>
-      </c>
-      <c r="F71" s="1">
-        <v>2.73</v>
-      </c>
-      <c r="G71" s="1">
-        <v>29.34</v>
-      </c>
-      <c r="I71" s="1">
-        <v>24.59</v>
-      </c>
-    </row>
-    <row r="72" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A72" t="s">
-        <v>164</v>
-      </c>
-      <c r="C72" t="str" cm="1">
-        <f t="array" ref="C72">_xlfn.IFS(
-ISNUMBER(SEARCH("IV*",A72)),"IV",
-ISNUMBER(SEARCH("III*",A72)),"III",
-ISNUMBER(SEARCH("II*",A72)),"II",
-ISNUMBER(SEARCH("I*",A72)),"I")</f>
-        <v>IV</v>
-      </c>
-      <c r="D72" cm="1">
-        <f t="array" ref="D72">_xlfn.IFS(
-ISNUMBER(SEARCH("-1*",A72)),1,
-ISNUMBER(SEARCH("-2*",A72)),2)</f>
-        <v>1</v>
-      </c>
-      <c r="E72" t="str" cm="1">
-        <f t="array" ref="E72">_xlfn.IFS(
-ISNUMBER(SEARCH("AUHV*",A72)),"AUHV",
-ISNUMBER(SEARCH("BWW*",A72)),"BWW",
-ISNUMBER(SEARCH("C1*",A72)),"C1",
-ISNUMBER(SEARCH("C2*",A72)),"C2",
-ISNUMBER(SEARCH("ORG*",A72)),"ORG",
-ISNUMBER(SEARCH("PRY*",A72)),"PRY",
-ISNUMBER(SEARCH("RCL*",A72)),"RCL",
-ISNUMBER(SEARCH("SWW*",A72)),"SWW",
-ISNUMBER(SEARCH("MNHV*",A72)),"MNHV")</f>
-        <v>SWW</v>
-      </c>
-      <c r="F72" s="1">
-        <v>2.75</v>
-      </c>
-      <c r="G72" s="1">
-        <v>28.72</v>
-      </c>
-      <c r="I72" s="1">
-        <v>23.47</v>
-      </c>
-    </row>
-    <row r="73" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A73" t="s">
-        <v>165</v>
-      </c>
-      <c r="C73" t="str" cm="1">
-        <f t="array" ref="C73">_xlfn.IFS(
-ISNUMBER(SEARCH("IV*",A73)),"IV",
-ISNUMBER(SEARCH("III*",A73)),"III",
-ISNUMBER(SEARCH("II*",A73)),"II",
-ISNUMBER(SEARCH("I*",A73)),"I")</f>
-        <v>IV</v>
-      </c>
-      <c r="D73" cm="1">
-        <f t="array" ref="D73">_xlfn.IFS(
-ISNUMBER(SEARCH("-1*",A73)),1,
-ISNUMBER(SEARCH("-2*",A73)),2)</f>
-        <v>2</v>
-      </c>
-      <c r="E73" t="str" cm="1">
-        <f t="array" ref="E73">_xlfn.IFS(
-ISNUMBER(SEARCH("AUHV*",A73)),"AUHV",
-ISNUMBER(SEARCH("BWW*",A73)),"BWW",
-ISNUMBER(SEARCH("C1*",A73)),"C1",
-ISNUMBER(SEARCH("C2*",A73)),"C2",
-ISNUMBER(SEARCH("ORG*",A73)),"ORG",
-ISNUMBER(SEARCH("PRY*",A73)),"PRY",
-ISNUMBER(SEARCH("RCL*",A73)),"RCL",
-ISNUMBER(SEARCH("SWW*",A73)),"SWW",
-ISNUMBER(SEARCH("MNHV*",A73)),"MNHV")</f>
-        <v>SWW</v>
-      </c>
-      <c r="F73" s="1">
-        <v>2.73</v>
-      </c>
-      <c r="G73" s="1">
+      <c r="G61" s="1">
         <v>28.14</v>
       </c>
-      <c r="I73" s="1">
+      <c r="H61">
+        <f t="shared" si="3"/>
+        <v>25.41</v>
+      </c>
+      <c r="I61" s="1">
         <v>23.03</v>
+      </c>
+      <c r="J61">
+        <f t="shared" si="4"/>
+        <v>20.3</v>
+      </c>
+      <c r="K61">
+        <f t="shared" si="5"/>
+        <v>79.889807162534439</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1271E86A-E210-4E47-AD27-BCA97BD73E7F}">
+  <dimension ref="A1:D2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="2" max="2" width="15.83203125" customWidth="1"/>
+    <col min="3" max="3" width="12.33203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>173</v>
+      </c>
+      <c r="B1" t="s">
+        <v>174</v>
+      </c>
+      <c r="C1" t="s">
+        <v>175</v>
+      </c>
+      <c r="D1" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A2">
+        <v>26.86</v>
+      </c>
+      <c r="B2">
+        <v>893.2</v>
+      </c>
+      <c r="C2">
+        <f>B2-A2</f>
+        <v>866.34</v>
+      </c>
+      <c r="D2" t="s">
+        <v>171</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>